<commit_message>
WIP：每小时保存全部进度 2026-09-17 22:55:14 -04:00
</commit_message>
<xml_diff>
--- a/data/Item.xlsx
+++ b/data/Item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,10 +432,22 @@
           <t>equip_kind</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>battle_usable</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>battle_heal_hp</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>battle_heal_mp</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
@@ -447,6 +459,21 @@
           <t>装备部位:0=不是装备。&gt;0=该部位编号。部位的含义(手镯/头/胸…)以及每个部位有几个槽,全部由数据定义 —— 槽位表 EquipSlot 决定哪个槽接受哪个部位,代码里不写死</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>回合制战斗内可用:0=不可用,1=可用</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>战斗内使用回复的生命值(0=不回血)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>战斗内使用回复的法力值(0=不回蓝)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -457,6 +484,15 @@
       </c>
       <c r="C6" t="n">
         <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -469,6 +505,15 @@
       <c r="C7" t="n">
         <v>1</v>
       </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -480,6 +525,15 @@
       <c r="C8" t="n">
         <v>0</v>
       </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -491,6 +545,15 @@
       <c r="C9" t="n">
         <v>0</v>
       </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -502,6 +565,15 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -513,6 +585,15 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -524,6 +605,15 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -535,6 +625,15 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -546,6 +645,15 @@
       <c r="C14" t="n">
         <v>0</v>
       </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -557,6 +665,15 @@
       <c r="C15" t="n">
         <v>0</v>
       </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>300</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -568,6 +685,15 @@
       <c r="C16" t="n">
         <v>0</v>
       </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -579,6 +705,15 @@
       <c r="C17" t="n">
         <v>0</v>
       </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -590,6 +725,15 @@
       <c r="C18" t="n">
         <v>0</v>
       </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -601,6 +745,15 @@
       <c r="C19" t="n">
         <v>0</v>
       </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -612,6 +765,15 @@
       <c r="C20" t="n">
         <v>0</v>
       </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -623,6 +785,15 @@
       <c r="C21" t="n">
         <v>0</v>
       </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -634,6 +805,15 @@
       <c r="C22" t="n">
         <v>0</v>
       </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -645,6 +825,15 @@
       <c r="C23" t="n">
         <v>0</v>
       </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -656,6 +845,15 @@
       <c r="C24" t="n">
         <v>0</v>
       </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -667,6 +865,15 @@
       <c r="C25" t="n">
         <v>0</v>
       </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -678,6 +885,15 @@
       <c r="C26" t="n">
         <v>0</v>
       </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -689,6 +905,15 @@
       <c r="C27" t="n">
         <v>0</v>
       </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -700,6 +925,15 @@
       <c r="C28" t="n">
         <v>0</v>
       </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -711,6 +945,15 @@
       <c r="C29" t="n">
         <v>0</v>
       </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -722,6 +965,15 @@
       <c r="C30" t="n">
         <v>0</v>
       </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -733,6 +985,15 @@
       <c r="C31" t="n">
         <v>0</v>
       </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -744,6 +1005,15 @@
       <c r="C32" t="n">
         <v>0</v>
       </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -753,6 +1023,15 @@
         <v>999</v>
       </c>
       <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>